<commit_message>
Label internal consistency coefficients explicitly as Pearson
</commit_message>
<xml_diff>
--- a/outputs/internal_consistency.xlsx
+++ b/outputs/internal_consistency.xlsx
@@ -590,8 +590,8 @@
     <col width="47" customWidth="1" min="2" max="2"/>
     <col width="13" customWidth="1" min="3" max="3"/>
     <col width="11" customWidth="1" min="4" max="4"/>
-    <col width="15" customWidth="1" min="5" max="5"/>
-    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="21" customWidth="1" min="5" max="5"/>
+    <col width="21" customWidth="1" min="6" max="6"/>
     <col width="19" customWidth="1" min="7" max="7"/>
     <col width="24" customWidth="1" min="8" max="8"/>
     <col width="17" customWidth="1" min="9" max="9"/>
@@ -648,12 +648,14 @@
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>أدنى r</t>
+          <t>أدنى معامل
+بيرسون المصحح r</t>
         </is>
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>أعلى r</t>
+          <t>أعلى معامل
+بيرسون المصحح r</t>
         </is>
       </c>
       <c r="G7" s="5" t="inlineStr">
@@ -1003,7 +1005,7 @@
     <col width="13" customWidth="1" min="1" max="1"/>
     <col width="88" customWidth="1" min="2" max="2"/>
     <col width="11" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="19" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="18" customWidth="1" min="6" max="6"/>
     <col width="19" customWidth="1" min="7" max="7"/>
@@ -1056,7 +1058,8 @@
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>r المصحح</t>
+          <t>معامل بيرسون
+المصحح r</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
@@ -1372,7 +1375,7 @@
     <col width="13" customWidth="1" min="1" max="1"/>
     <col width="88" customWidth="1" min="2" max="2"/>
     <col width="11" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="19" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="18" customWidth="1" min="6" max="6"/>
     <col width="19" customWidth="1" min="7" max="7"/>
@@ -1425,7 +1428,8 @@
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>r المصحح</t>
+          <t>معامل بيرسون
+المصحح r</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
@@ -1775,7 +1779,7 @@
     <col width="13" customWidth="1" min="1" max="1"/>
     <col width="88" customWidth="1" min="2" max="2"/>
     <col width="11" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="19" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="18" customWidth="1" min="6" max="6"/>
     <col width="19" customWidth="1" min="7" max="7"/>
@@ -1828,7 +1832,8 @@
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>r المصحح</t>
+          <t>معامل بيرسون
+المصحح r</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
@@ -2110,7 +2115,7 @@
     <col width="13" customWidth="1" min="1" max="1"/>
     <col width="88" customWidth="1" min="2" max="2"/>
     <col width="11" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="19" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="18" customWidth="1" min="6" max="6"/>
     <col width="19" customWidth="1" min="7" max="7"/>
@@ -2163,7 +2168,8 @@
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>r المصحح</t>
+          <t>معامل بيرسون
+المصحح r</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
@@ -2513,7 +2519,7 @@
     <col width="13" customWidth="1" min="1" max="1"/>
     <col width="88" customWidth="1" min="2" max="2"/>
     <col width="11" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="19" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="18" customWidth="1" min="6" max="6"/>
     <col width="19" customWidth="1" min="7" max="7"/>
@@ -2566,7 +2572,8 @@
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>r المصحح</t>
+          <t>معامل بيرسون
+المصحح r</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
@@ -2984,7 +2991,7 @@
     <col width="13" customWidth="1" min="1" max="1"/>
     <col width="88" customWidth="1" min="2" max="2"/>
     <col width="11" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="19" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="18" customWidth="1" min="6" max="6"/>
     <col width="19" customWidth="1" min="7" max="7"/>
@@ -3037,7 +3044,8 @@
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>r المصحح</t>
+          <t>معامل بيرسون
+المصحح r</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
@@ -3480,7 +3488,8 @@
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>r المصحح — دقيق</t>
+          <t>معامل بيرسون
+المصحح r — دقيق</t>
         </is>
       </c>
       <c r="F7" s="5" t="inlineStr">

</xml_diff>